<commit_message>
fix naik kelas, fix kelola anggota, fix tanggal masuk dan tanggal lahir import dan data siswa
</commit_message>
<xml_diff>
--- a/import/template-import-siswa.xlsx
+++ b/import/template-import-siswa.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30405"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11012"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\GodBoy\Documents\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/godboy/Project/nextjs/clone-rapor-next/import/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8285472C-AFBD-4906-884B-69A534CE87C7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A17D6318-4765-BC47-98C3-4D289931D40E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="920" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Template" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1165" uniqueCount="425">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1165" uniqueCount="426">
   <si>
     <t>Nama Siswa *</t>
   </si>
@@ -1309,6 +1309,9 @@
   </si>
   <si>
     <t>0112623469</t>
+  </si>
+  <si>
+    <t>X RPL</t>
   </si>
 </sst>
 </file>
@@ -1346,8 +1349,8 @@
   </cellStyleXfs>
   <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1688,21 +1691,21 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:O180"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="20.875" customWidth="1"/>
-    <col min="2" max="2" width="10.875" customWidth="1"/>
-    <col min="3" max="6" width="15.875" customWidth="1"/>
-    <col min="7" max="7" width="12.875" customWidth="1"/>
-    <col min="8" max="8" width="20.875" customWidth="1"/>
-    <col min="9" max="9" width="15.875" customWidth="1"/>
-    <col min="10" max="10" width="30.875" customWidth="1"/>
-    <col min="11" max="12" width="15.875" customWidth="1"/>
-    <col min="13" max="13" width="10.875" customWidth="1"/>
-    <col min="14" max="15" width="15.875" customWidth="1"/>
+    <col min="1" max="1" width="20.83203125" customWidth="1"/>
+    <col min="2" max="2" width="10.83203125" customWidth="1"/>
+    <col min="3" max="6" width="15.83203125" customWidth="1"/>
+    <col min="7" max="7" width="12.83203125" customWidth="1"/>
+    <col min="8" max="8" width="20.83203125" customWidth="1"/>
+    <col min="9" max="9" width="15.83203125" customWidth="1"/>
+    <col min="10" max="10" width="30.83203125" customWidth="1"/>
+    <col min="11" max="12" width="15.83203125" customWidth="1"/>
+    <col min="13" max="13" width="10.83203125" customWidth="1"/>
+    <col min="14" max="15" width="15.83203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1749,7 +1752,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="2" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>64</v>
       </c>
@@ -1759,7 +1762,7 @@
       <c r="K2" t="s">
         <v>136</v>
       </c>
-      <c r="L2" s="2">
+      <c r="L2" s="1">
         <v>46216</v>
       </c>
       <c r="M2" t="s">
@@ -1772,7 +1775,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="3" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>65</v>
       </c>
@@ -1782,7 +1785,7 @@
       <c r="K3" t="s">
         <v>136</v>
       </c>
-      <c r="L3" s="2">
+      <c r="L3" s="1">
         <v>46216</v>
       </c>
       <c r="M3" t="s">
@@ -1795,7 +1798,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="4" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>66</v>
       </c>
@@ -1805,7 +1808,7 @@
       <c r="K4" t="s">
         <v>136</v>
       </c>
-      <c r="L4" s="2">
+      <c r="L4" s="1">
         <v>46216</v>
       </c>
       <c r="M4" t="s">
@@ -1818,7 +1821,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="5" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>67</v>
       </c>
@@ -1828,7 +1831,7 @@
       <c r="K5" t="s">
         <v>136</v>
       </c>
-      <c r="L5" s="2">
+      <c r="L5" s="1">
         <v>46216</v>
       </c>
       <c r="M5" t="s">
@@ -1841,7 +1844,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="6" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>68</v>
       </c>
@@ -1851,7 +1854,7 @@
       <c r="K6" t="s">
         <v>136</v>
       </c>
-      <c r="L6" s="2">
+      <c r="L6" s="1">
         <v>46216</v>
       </c>
       <c r="M6" t="s">
@@ -1864,7 +1867,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="7" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>69</v>
       </c>
@@ -1874,7 +1877,7 @@
       <c r="K7" t="s">
         <v>136</v>
       </c>
-      <c r="L7" s="2">
+      <c r="L7" s="1">
         <v>46216</v>
       </c>
       <c r="M7" t="s">
@@ -1887,7 +1890,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="8" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>70</v>
       </c>
@@ -1897,7 +1900,7 @@
       <c r="K8" t="s">
         <v>136</v>
       </c>
-      <c r="L8" s="2">
+      <c r="L8" s="1">
         <v>46216</v>
       </c>
       <c r="M8" t="s">
@@ -1910,7 +1913,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="9" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>71</v>
       </c>
@@ -1920,7 +1923,7 @@
       <c r="K9" t="s">
         <v>136</v>
       </c>
-      <c r="L9" s="2">
+      <c r="L9" s="1">
         <v>46216</v>
       </c>
       <c r="M9" t="s">
@@ -1933,7 +1936,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="10" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>72</v>
       </c>
@@ -1943,7 +1946,7 @@
       <c r="K10" t="s">
         <v>136</v>
       </c>
-      <c r="L10" s="2">
+      <c r="L10" s="1">
         <v>46216</v>
       </c>
       <c r="M10" t="s">
@@ -1956,7 +1959,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="11" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>73</v>
       </c>
@@ -1966,7 +1969,7 @@
       <c r="K11" t="s">
         <v>136</v>
       </c>
-      <c r="L11" s="2">
+      <c r="L11" s="1">
         <v>46216</v>
       </c>
       <c r="M11" t="s">
@@ -1979,7 +1982,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="12" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>74</v>
       </c>
@@ -1989,7 +1992,7 @@
       <c r="K12" t="s">
         <v>136</v>
       </c>
-      <c r="L12" s="2">
+      <c r="L12" s="1">
         <v>46216</v>
       </c>
       <c r="M12" t="s">
@@ -2002,7 +2005,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="13" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
         <v>75</v>
       </c>
@@ -2012,7 +2015,7 @@
       <c r="K13" t="s">
         <v>136</v>
       </c>
-      <c r="L13" s="2">
+      <c r="L13" s="1">
         <v>46216</v>
       </c>
       <c r="M13" t="s">
@@ -2025,7 +2028,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="14" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
         <v>76</v>
       </c>
@@ -2035,7 +2038,7 @@
       <c r="K14" t="s">
         <v>136</v>
       </c>
-      <c r="L14" s="2">
+      <c r="L14" s="1">
         <v>46216</v>
       </c>
       <c r="M14" t="s">
@@ -2048,7 +2051,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="15" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
         <v>77</v>
       </c>
@@ -2058,7 +2061,7 @@
       <c r="K15" t="s">
         <v>136</v>
       </c>
-      <c r="L15" s="2">
+      <c r="L15" s="1">
         <v>46216</v>
       </c>
       <c r="M15" t="s">
@@ -2071,7 +2074,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="16" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
         <v>78</v>
       </c>
@@ -2081,7 +2084,7 @@
       <c r="K16" t="s">
         <v>136</v>
       </c>
-      <c r="L16" s="2">
+      <c r="L16" s="1">
         <v>46216</v>
       </c>
       <c r="M16" t="s">
@@ -2094,7 +2097,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="17" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
         <v>79</v>
       </c>
@@ -2104,7 +2107,7 @@
       <c r="K17" t="s">
         <v>136</v>
       </c>
-      <c r="L17" s="2">
+      <c r="L17" s="1">
         <v>46216</v>
       </c>
       <c r="M17" t="s">
@@ -2117,7 +2120,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="18" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
         <v>80</v>
       </c>
@@ -2127,7 +2130,7 @@
       <c r="K18" t="s">
         <v>136</v>
       </c>
-      <c r="L18" s="2">
+      <c r="L18" s="1">
         <v>46216</v>
       </c>
       <c r="M18" t="s">
@@ -2140,7 +2143,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="19" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
         <v>81</v>
       </c>
@@ -2150,7 +2153,7 @@
       <c r="K19" t="s">
         <v>136</v>
       </c>
-      <c r="L19" s="2">
+      <c r="L19" s="1">
         <v>46216</v>
       </c>
       <c r="M19" t="s">
@@ -2163,7 +2166,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="20" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
         <v>82</v>
       </c>
@@ -2173,7 +2176,7 @@
       <c r="K20" t="s">
         <v>136</v>
       </c>
-      <c r="L20" s="2">
+      <c r="L20" s="1">
         <v>46216</v>
       </c>
       <c r="M20" t="s">
@@ -2186,7 +2189,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="21" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
         <v>83</v>
       </c>
@@ -2196,7 +2199,7 @@
       <c r="K21" t="s">
         <v>136</v>
       </c>
-      <c r="L21" s="2">
+      <c r="L21" s="1">
         <v>46216</v>
       </c>
       <c r="M21" t="s">
@@ -2209,7 +2212,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="22" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
         <v>84</v>
       </c>
@@ -2219,7 +2222,7 @@
       <c r="K22" t="s">
         <v>136</v>
       </c>
-      <c r="L22" s="2">
+      <c r="L22" s="1">
         <v>46216</v>
       </c>
       <c r="M22" t="s">
@@ -2232,7 +2235,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="23" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
         <v>85</v>
       </c>
@@ -2242,7 +2245,7 @@
       <c r="K23" t="s">
         <v>136</v>
       </c>
-      <c r="L23" s="2">
+      <c r="L23" s="1">
         <v>46216</v>
       </c>
       <c r="M23" t="s">
@@ -2255,7 +2258,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="24" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
         <v>86</v>
       </c>
@@ -2265,7 +2268,7 @@
       <c r="K24" t="s">
         <v>136</v>
       </c>
-      <c r="L24" s="2">
+      <c r="L24" s="1">
         <v>46216</v>
       </c>
       <c r="M24" t="s">
@@ -2278,7 +2281,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="25" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
         <v>87</v>
       </c>
@@ -2288,7 +2291,7 @@
       <c r="K25" t="s">
         <v>136</v>
       </c>
-      <c r="L25" s="2">
+      <c r="L25" s="1">
         <v>46216</v>
       </c>
       <c r="M25" t="s">
@@ -2301,7 +2304,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="26" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
         <v>88</v>
       </c>
@@ -2311,7 +2314,7 @@
       <c r="K26" t="s">
         <v>136</v>
       </c>
-      <c r="L26" s="2">
+      <c r="L26" s="1">
         <v>46216</v>
       </c>
       <c r="M26" t="s">
@@ -2324,7 +2327,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="27" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
         <v>89</v>
       </c>
@@ -2334,7 +2337,7 @@
       <c r="K27" t="s">
         <v>136</v>
       </c>
-      <c r="L27" s="2">
+      <c r="L27" s="1">
         <v>46216</v>
       </c>
       <c r="M27" t="s">
@@ -2347,7 +2350,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="28" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
         <v>90</v>
       </c>
@@ -2357,7 +2360,7 @@
       <c r="K28" t="s">
         <v>136</v>
       </c>
-      <c r="L28" s="2">
+      <c r="L28" s="1">
         <v>46216</v>
       </c>
       <c r="M28" t="s">
@@ -2370,7 +2373,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="29" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
         <v>91</v>
       </c>
@@ -2380,7 +2383,7 @@
       <c r="K29" t="s">
         <v>136</v>
       </c>
-      <c r="L29" s="2">
+      <c r="L29" s="1">
         <v>46216</v>
       </c>
       <c r="M29" t="s">
@@ -2393,7 +2396,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="30" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
         <v>92</v>
       </c>
@@ -2403,7 +2406,7 @@
       <c r="K30" t="s">
         <v>136</v>
       </c>
-      <c r="L30" s="2">
+      <c r="L30" s="1">
         <v>46216</v>
       </c>
       <c r="M30" t="s">
@@ -2416,7 +2419,7 @@
         <v>128</v>
       </c>
     </row>
-    <row r="31" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
         <v>93</v>
       </c>
@@ -2426,7 +2429,7 @@
       <c r="K31" t="s">
         <v>136</v>
       </c>
-      <c r="L31" s="2">
+      <c r="L31" s="1">
         <v>46216</v>
       </c>
       <c r="M31" t="s">
@@ -2439,7 +2442,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="32" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
         <v>94</v>
       </c>
@@ -2449,7 +2452,7 @@
       <c r="K32" t="s">
         <v>136</v>
       </c>
-      <c r="L32" s="2">
+      <c r="L32" s="1">
         <v>46216</v>
       </c>
       <c r="M32" t="s">
@@ -2462,7 +2465,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="33" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
         <v>95</v>
       </c>
@@ -2472,7 +2475,7 @@
       <c r="K33" t="s">
         <v>136</v>
       </c>
-      <c r="L33" s="2">
+      <c r="L33" s="1">
         <v>46216</v>
       </c>
       <c r="M33" t="s">
@@ -2485,7 +2488,7 @@
         <v>131</v>
       </c>
     </row>
-    <row r="34" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
         <v>96</v>
       </c>
@@ -2495,7 +2498,7 @@
       <c r="K34" t="s">
         <v>136</v>
       </c>
-      <c r="L34" s="2">
+      <c r="L34" s="1">
         <v>46216</v>
       </c>
       <c r="M34" t="s">
@@ -2508,7 +2511,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="35" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
         <v>97</v>
       </c>
@@ -2518,7 +2521,7 @@
       <c r="K35" t="s">
         <v>136</v>
       </c>
-      <c r="L35" s="2">
+      <c r="L35" s="1">
         <v>46216</v>
       </c>
       <c r="M35" t="s">
@@ -2531,7 +2534,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="36" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
         <v>98</v>
       </c>
@@ -2541,7 +2544,7 @@
       <c r="K36" t="s">
         <v>136</v>
       </c>
-      <c r="L36" s="2">
+      <c r="L36" s="1">
         <v>46216</v>
       </c>
       <c r="M36" t="s">
@@ -2554,7 +2557,7 @@
         <v>134</v>
       </c>
     </row>
-    <row r="37" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
         <v>99</v>
       </c>
@@ -2564,7 +2567,7 @@
       <c r="K37" t="s">
         <v>136</v>
       </c>
-      <c r="L37" s="2">
+      <c r="L37" s="1">
         <v>46216</v>
       </c>
       <c r="M37" t="s">
@@ -2577,7 +2580,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="38" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
         <v>137</v>
       </c>
@@ -2587,7 +2590,7 @@
       <c r="K38" t="s">
         <v>173</v>
       </c>
-      <c r="L38" s="2">
+      <c r="L38" s="1">
         <v>46216</v>
       </c>
       <c r="M38" t="s">
@@ -2600,7 +2603,7 @@
         <v>174</v>
       </c>
     </row>
-    <row r="39" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
         <v>138</v>
       </c>
@@ -2610,7 +2613,7 @@
       <c r="K39" t="s">
         <v>173</v>
       </c>
-      <c r="L39" s="2">
+      <c r="L39" s="1">
         <v>46216</v>
       </c>
       <c r="M39" t="s">
@@ -2623,7 +2626,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="40" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
         <v>139</v>
       </c>
@@ -2633,7 +2636,7 @@
       <c r="K40" t="s">
         <v>173</v>
       </c>
-      <c r="L40" s="2">
+      <c r="L40" s="1">
         <v>46216</v>
       </c>
       <c r="M40" t="s">
@@ -2646,7 +2649,7 @@
         <v>176</v>
       </c>
     </row>
-    <row r="41" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
         <v>140</v>
       </c>
@@ -2656,7 +2659,7 @@
       <c r="K41" t="s">
         <v>173</v>
       </c>
-      <c r="L41" s="2">
+      <c r="L41" s="1">
         <v>46216</v>
       </c>
       <c r="M41" t="s">
@@ -2669,7 +2672,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="42" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
         <v>141</v>
       </c>
@@ -2679,7 +2682,7 @@
       <c r="K42" t="s">
         <v>173</v>
       </c>
-      <c r="L42" s="2">
+      <c r="L42" s="1">
         <v>46216</v>
       </c>
       <c r="M42" t="s">
@@ -2692,7 +2695,7 @@
         <v>178</v>
       </c>
     </row>
-    <row r="43" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A43" t="s">
         <v>142</v>
       </c>
@@ -2702,7 +2705,7 @@
       <c r="K43" t="s">
         <v>173</v>
       </c>
-      <c r="L43" s="2">
+      <c r="L43" s="1">
         <v>46216</v>
       </c>
       <c r="M43" t="s">
@@ -2715,7 +2718,7 @@
         <v>179</v>
       </c>
     </row>
-    <row r="44" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A44" t="s">
         <v>143</v>
       </c>
@@ -2725,7 +2728,7 @@
       <c r="K44" t="s">
         <v>173</v>
       </c>
-      <c r="L44" s="2">
+      <c r="L44" s="1">
         <v>46216</v>
       </c>
       <c r="M44" t="s">
@@ -2738,7 +2741,7 @@
         <v>180</v>
       </c>
     </row>
-    <row r="45" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A45" t="s">
         <v>144</v>
       </c>
@@ -2748,7 +2751,7 @@
       <c r="K45" t="s">
         <v>173</v>
       </c>
-      <c r="L45" s="2">
+      <c r="L45" s="1">
         <v>46216</v>
       </c>
       <c r="M45" t="s">
@@ -2761,7 +2764,7 @@
         <v>181</v>
       </c>
     </row>
-    <row r="46" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A46" t="s">
         <v>145</v>
       </c>
@@ -2771,7 +2774,7 @@
       <c r="K46" t="s">
         <v>173</v>
       </c>
-      <c r="L46" s="2">
+      <c r="L46" s="1">
         <v>46216</v>
       </c>
       <c r="M46" t="s">
@@ -2784,7 +2787,7 @@
         <v>182</v>
       </c>
     </row>
-    <row r="47" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A47" t="s">
         <v>146</v>
       </c>
@@ -2794,7 +2797,7 @@
       <c r="K47" t="s">
         <v>173</v>
       </c>
-      <c r="L47" s="2">
+      <c r="L47" s="1">
         <v>46216</v>
       </c>
       <c r="M47" t="s">
@@ -2807,7 +2810,7 @@
         <v>183</v>
       </c>
     </row>
-    <row r="48" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A48" t="s">
         <v>147</v>
       </c>
@@ -2817,7 +2820,7 @@
       <c r="K48" t="s">
         <v>173</v>
       </c>
-      <c r="L48" s="2">
+      <c r="L48" s="1">
         <v>46216</v>
       </c>
       <c r="M48" t="s">
@@ -2830,7 +2833,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="49" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A49" t="s">
         <v>148</v>
       </c>
@@ -2840,7 +2843,7 @@
       <c r="K49" t="s">
         <v>173</v>
       </c>
-      <c r="L49" s="2">
+      <c r="L49" s="1">
         <v>46216</v>
       </c>
       <c r="M49" t="s">
@@ -2853,7 +2856,7 @@
         <v>185</v>
       </c>
     </row>
-    <row r="50" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A50" t="s">
         <v>149</v>
       </c>
@@ -2863,7 +2866,7 @@
       <c r="K50" t="s">
         <v>173</v>
       </c>
-      <c r="L50" s="2">
+      <c r="L50" s="1">
         <v>46216</v>
       </c>
       <c r="M50" t="s">
@@ -2876,7 +2879,7 @@
         <v>186</v>
       </c>
     </row>
-    <row r="51" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A51" t="s">
         <v>150</v>
       </c>
@@ -2886,7 +2889,7 @@
       <c r="K51" t="s">
         <v>173</v>
       </c>
-      <c r="L51" s="2">
+      <c r="L51" s="1">
         <v>46216</v>
       </c>
       <c r="M51" t="s">
@@ -2899,7 +2902,7 @@
         <v>187</v>
       </c>
     </row>
-    <row r="52" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A52" t="s">
         <v>151</v>
       </c>
@@ -2909,7 +2912,7 @@
       <c r="K52" t="s">
         <v>173</v>
       </c>
-      <c r="L52" s="2">
+      <c r="L52" s="1">
         <v>46216</v>
       </c>
       <c r="M52" t="s">
@@ -2922,7 +2925,7 @@
         <v>188</v>
       </c>
     </row>
-    <row r="53" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A53" t="s">
         <v>152</v>
       </c>
@@ -2932,7 +2935,7 @@
       <c r="K53" t="s">
         <v>173</v>
       </c>
-      <c r="L53" s="2">
+      <c r="L53" s="1">
         <v>46216</v>
       </c>
       <c r="M53" t="s">
@@ -2945,7 +2948,7 @@
         <v>189</v>
       </c>
     </row>
-    <row r="54" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A54" t="s">
         <v>153</v>
       </c>
@@ -2955,7 +2958,7 @@
       <c r="K54" t="s">
         <v>173</v>
       </c>
-      <c r="L54" s="2">
+      <c r="L54" s="1">
         <v>46216</v>
       </c>
       <c r="M54" t="s">
@@ -2968,7 +2971,7 @@
         <v>190</v>
       </c>
     </row>
-    <row r="55" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A55" t="s">
         <v>154</v>
       </c>
@@ -2978,7 +2981,7 @@
       <c r="K55" t="s">
         <v>173</v>
       </c>
-      <c r="L55" s="2">
+      <c r="L55" s="1">
         <v>46216</v>
       </c>
       <c r="M55" t="s">
@@ -2991,7 +2994,7 @@
         <v>191</v>
       </c>
     </row>
-    <row r="56" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A56" t="s">
         <v>155</v>
       </c>
@@ -3001,7 +3004,7 @@
       <c r="K56" t="s">
         <v>173</v>
       </c>
-      <c r="L56" s="2">
+      <c r="L56" s="1">
         <v>46216</v>
       </c>
       <c r="M56" t="s">
@@ -3014,7 +3017,7 @@
         <v>192</v>
       </c>
     </row>
-    <row r="57" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A57" t="s">
         <v>156</v>
       </c>
@@ -3024,7 +3027,7 @@
       <c r="K57" t="s">
         <v>173</v>
       </c>
-      <c r="L57" s="2">
+      <c r="L57" s="1">
         <v>46216</v>
       </c>
       <c r="M57" t="s">
@@ -3037,7 +3040,7 @@
         <v>193</v>
       </c>
     </row>
-    <row r="58" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A58" t="s">
         <v>157</v>
       </c>
@@ -3047,7 +3050,7 @@
       <c r="K58" t="s">
         <v>173</v>
       </c>
-      <c r="L58" s="2">
+      <c r="L58" s="1">
         <v>46216</v>
       </c>
       <c r="M58" t="s">
@@ -3060,7 +3063,7 @@
         <v>194</v>
       </c>
     </row>
-    <row r="59" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A59" t="s">
         <v>158</v>
       </c>
@@ -3070,7 +3073,7 @@
       <c r="K59" t="s">
         <v>173</v>
       </c>
-      <c r="L59" s="2">
+      <c r="L59" s="1">
         <v>46216</v>
       </c>
       <c r="M59" t="s">
@@ -3083,7 +3086,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="60" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A60" t="s">
         <v>159</v>
       </c>
@@ -3093,7 +3096,7 @@
       <c r="K60" t="s">
         <v>173</v>
       </c>
-      <c r="L60" s="2">
+      <c r="L60" s="1">
         <v>46216</v>
       </c>
       <c r="M60" t="s">
@@ -3106,7 +3109,7 @@
         <v>196</v>
       </c>
     </row>
-    <row r="61" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A61" t="s">
         <v>160</v>
       </c>
@@ -3116,7 +3119,7 @@
       <c r="K61" t="s">
         <v>173</v>
       </c>
-      <c r="L61" s="2">
+      <c r="L61" s="1">
         <v>46216</v>
       </c>
       <c r="M61" t="s">
@@ -3129,7 +3132,7 @@
         <v>197</v>
       </c>
     </row>
-    <row r="62" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A62" t="s">
         <v>161</v>
       </c>
@@ -3139,7 +3142,7 @@
       <c r="K62" t="s">
         <v>173</v>
       </c>
-      <c r="L62" s="2">
+      <c r="L62" s="1">
         <v>46216</v>
       </c>
       <c r="M62" t="s">
@@ -3152,7 +3155,7 @@
         <v>198</v>
       </c>
     </row>
-    <row r="63" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A63" t="s">
         <v>162</v>
       </c>
@@ -3162,7 +3165,7 @@
       <c r="K63" t="s">
         <v>173</v>
       </c>
-      <c r="L63" s="2">
+      <c r="L63" s="1">
         <v>46216</v>
       </c>
       <c r="M63" t="s">
@@ -3175,7 +3178,7 @@
         <v>199</v>
       </c>
     </row>
-    <row r="64" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A64" t="s">
         <v>163</v>
       </c>
@@ -3185,7 +3188,7 @@
       <c r="K64" t="s">
         <v>173</v>
       </c>
-      <c r="L64" s="2">
+      <c r="L64" s="1">
         <v>46216</v>
       </c>
       <c r="M64" t="s">
@@ -3198,7 +3201,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="65" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A65" t="s">
         <v>164</v>
       </c>
@@ -3208,7 +3211,7 @@
       <c r="K65" t="s">
         <v>173</v>
       </c>
-      <c r="L65" s="2">
+      <c r="L65" s="1">
         <v>46216</v>
       </c>
       <c r="M65" t="s">
@@ -3221,7 +3224,7 @@
         <v>201</v>
       </c>
     </row>
-    <row r="66" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A66" t="s">
         <v>165</v>
       </c>
@@ -3231,7 +3234,7 @@
       <c r="K66" t="s">
         <v>173</v>
       </c>
-      <c r="L66" s="2">
+      <c r="L66" s="1">
         <v>46216</v>
       </c>
       <c r="M66" t="s">
@@ -3244,7 +3247,7 @@
         <v>202</v>
       </c>
     </row>
-    <row r="67" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A67" t="s">
         <v>166</v>
       </c>
@@ -3254,7 +3257,7 @@
       <c r="K67" t="s">
         <v>173</v>
       </c>
-      <c r="L67" s="2">
+      <c r="L67" s="1">
         <v>46216</v>
       </c>
       <c r="M67" t="s">
@@ -3267,7 +3270,7 @@
         <v>203</v>
       </c>
     </row>
-    <row r="68" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A68" t="s">
         <v>167</v>
       </c>
@@ -3277,7 +3280,7 @@
       <c r="K68" t="s">
         <v>173</v>
       </c>
-      <c r="L68" s="2">
+      <c r="L68" s="1">
         <v>46216</v>
       </c>
       <c r="M68" t="s">
@@ -3290,7 +3293,7 @@
         <v>204</v>
       </c>
     </row>
-    <row r="69" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A69" t="s">
         <v>168</v>
       </c>
@@ -3300,7 +3303,7 @@
       <c r="K69" t="s">
         <v>173</v>
       </c>
-      <c r="L69" s="2">
+      <c r="L69" s="1">
         <v>46216</v>
       </c>
       <c r="M69" t="s">
@@ -3313,7 +3316,7 @@
         <v>205</v>
       </c>
     </row>
-    <row r="70" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A70" t="s">
         <v>169</v>
       </c>
@@ -3323,7 +3326,7 @@
       <c r="K70" t="s">
         <v>173</v>
       </c>
-      <c r="L70" s="2">
+      <c r="L70" s="1">
         <v>46216</v>
       </c>
       <c r="M70" t="s">
@@ -3336,7 +3339,7 @@
         <v>206</v>
       </c>
     </row>
-    <row r="71" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A71" t="s">
         <v>170</v>
       </c>
@@ -3346,7 +3349,7 @@
       <c r="K71" t="s">
         <v>173</v>
       </c>
-      <c r="L71" s="2">
+      <c r="L71" s="1">
         <v>46216</v>
       </c>
       <c r="M71" t="s">
@@ -3359,7 +3362,7 @@
         <v>207</v>
       </c>
     </row>
-    <row r="72" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A72" t="s">
         <v>171</v>
       </c>
@@ -3369,7 +3372,7 @@
       <c r="K72" t="s">
         <v>173</v>
       </c>
-      <c r="L72" s="2">
+      <c r="L72" s="1">
         <v>46216</v>
       </c>
       <c r="M72" t="s">
@@ -3382,7 +3385,7 @@
         <v>208</v>
       </c>
     </row>
-    <row r="73" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A73" t="s">
         <v>172</v>
       </c>
@@ -3392,7 +3395,7 @@
       <c r="K73" t="s">
         <v>173</v>
       </c>
-      <c r="L73" s="2">
+      <c r="L73" s="1">
         <v>46216</v>
       </c>
       <c r="M73" t="s">
@@ -3405,7 +3408,7 @@
         <v>209</v>
       </c>
     </row>
-    <row r="74" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A74" t="s">
         <v>247</v>
       </c>
@@ -3415,7 +3418,7 @@
       <c r="K74" t="s">
         <v>246</v>
       </c>
-      <c r="L74" s="2">
+      <c r="L74" s="1">
         <v>46216</v>
       </c>
       <c r="M74" t="s">
@@ -3428,7 +3431,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="75" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A75" t="s">
         <v>248</v>
       </c>
@@ -3438,7 +3441,7 @@
       <c r="K75" t="s">
         <v>246</v>
       </c>
-      <c r="L75" s="2">
+      <c r="L75" s="1">
         <v>46216</v>
       </c>
       <c r="M75" t="s">
@@ -3451,7 +3454,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="76" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A76" t="s">
         <v>249</v>
       </c>
@@ -3461,7 +3464,7 @@
       <c r="K76" t="s">
         <v>246</v>
       </c>
-      <c r="L76" s="2">
+      <c r="L76" s="1">
         <v>46216</v>
       </c>
       <c r="M76" t="s">
@@ -3474,7 +3477,7 @@
         <v>212</v>
       </c>
     </row>
-    <row r="77" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A77" t="s">
         <v>250</v>
       </c>
@@ -3484,7 +3487,7 @@
       <c r="K77" t="s">
         <v>246</v>
       </c>
-      <c r="L77" s="2">
+      <c r="L77" s="1">
         <v>46216</v>
       </c>
       <c r="M77" t="s">
@@ -3497,7 +3500,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="78" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A78" t="s">
         <v>251</v>
       </c>
@@ -3507,7 +3510,7 @@
       <c r="K78" t="s">
         <v>246</v>
       </c>
-      <c r="L78" s="2">
+      <c r="L78" s="1">
         <v>46216</v>
       </c>
       <c r="M78" t="s">
@@ -3520,7 +3523,7 @@
         <v>214</v>
       </c>
     </row>
-    <row r="79" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A79" t="s">
         <v>252</v>
       </c>
@@ -3530,7 +3533,7 @@
       <c r="K79" t="s">
         <v>246</v>
       </c>
-      <c r="L79" s="2">
+      <c r="L79" s="1">
         <v>46216</v>
       </c>
       <c r="M79" t="s">
@@ -3543,7 +3546,7 @@
         <v>215</v>
       </c>
     </row>
-    <row r="80" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A80" t="s">
         <v>253</v>
       </c>
@@ -3553,7 +3556,7 @@
       <c r="K80" t="s">
         <v>246</v>
       </c>
-      <c r="L80" s="2">
+      <c r="L80" s="1">
         <v>46216</v>
       </c>
       <c r="M80" t="s">
@@ -3566,7 +3569,7 @@
         <v>216</v>
       </c>
     </row>
-    <row r="81" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A81" t="s">
         <v>254</v>
       </c>
@@ -3576,7 +3579,7 @@
       <c r="K81" t="s">
         <v>246</v>
       </c>
-      <c r="L81" s="2">
+      <c r="L81" s="1">
         <v>46216</v>
       </c>
       <c r="M81" t="s">
@@ -3589,7 +3592,7 @@
         <v>217</v>
       </c>
     </row>
-    <row r="82" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A82" t="s">
         <v>255</v>
       </c>
@@ -3599,7 +3602,7 @@
       <c r="K82" t="s">
         <v>246</v>
       </c>
-      <c r="L82" s="2">
+      <c r="L82" s="1">
         <v>46216</v>
       </c>
       <c r="M82" t="s">
@@ -3612,7 +3615,7 @@
         <v>218</v>
       </c>
     </row>
-    <row r="83" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A83" t="s">
         <v>256</v>
       </c>
@@ -3622,7 +3625,7 @@
       <c r="K83" t="s">
         <v>246</v>
       </c>
-      <c r="L83" s="2">
+      <c r="L83" s="1">
         <v>46216</v>
       </c>
       <c r="M83" t="s">
@@ -3635,7 +3638,7 @@
         <v>219</v>
       </c>
     </row>
-    <row r="84" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A84" t="s">
         <v>257</v>
       </c>
@@ -3645,7 +3648,7 @@
       <c r="K84" t="s">
         <v>246</v>
       </c>
-      <c r="L84" s="2">
+      <c r="L84" s="1">
         <v>46216</v>
       </c>
       <c r="M84" t="s">
@@ -3658,7 +3661,7 @@
         <v>220</v>
       </c>
     </row>
-    <row r="85" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A85" t="s">
         <v>258</v>
       </c>
@@ -3668,7 +3671,7 @@
       <c r="K85" t="s">
         <v>246</v>
       </c>
-      <c r="L85" s="2">
+      <c r="L85" s="1">
         <v>46216</v>
       </c>
       <c r="M85" t="s">
@@ -3681,7 +3684,7 @@
         <v>221</v>
       </c>
     </row>
-    <row r="86" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A86" t="s">
         <v>259</v>
       </c>
@@ -3691,7 +3694,7 @@
       <c r="K86" t="s">
         <v>246</v>
       </c>
-      <c r="L86" s="2">
+      <c r="L86" s="1">
         <v>46216</v>
       </c>
       <c r="M86" t="s">
@@ -3704,7 +3707,7 @@
         <v>222</v>
       </c>
     </row>
-    <row r="87" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A87" t="s">
         <v>260</v>
       </c>
@@ -3714,7 +3717,7 @@
       <c r="K87" t="s">
         <v>246</v>
       </c>
-      <c r="L87" s="2">
+      <c r="L87" s="1">
         <v>46216</v>
       </c>
       <c r="M87" t="s">
@@ -3727,7 +3730,7 @@
         <v>223</v>
       </c>
     </row>
-    <row r="88" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A88" t="s">
         <v>261</v>
       </c>
@@ -3737,7 +3740,7 @@
       <c r="K88" t="s">
         <v>246</v>
       </c>
-      <c r="L88" s="2">
+      <c r="L88" s="1">
         <v>46216</v>
       </c>
       <c r="M88" t="s">
@@ -3750,7 +3753,7 @@
         <v>224</v>
       </c>
     </row>
-    <row r="89" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A89" t="s">
         <v>262</v>
       </c>
@@ -3760,7 +3763,7 @@
       <c r="K89" t="s">
         <v>246</v>
       </c>
-      <c r="L89" s="2">
+      <c r="L89" s="1">
         <v>46216</v>
       </c>
       <c r="M89" t="s">
@@ -3773,7 +3776,7 @@
         <v>225</v>
       </c>
     </row>
-    <row r="90" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A90" t="s">
         <v>263</v>
       </c>
@@ -3783,7 +3786,7 @@
       <c r="K90" t="s">
         <v>246</v>
       </c>
-      <c r="L90" s="2">
+      <c r="L90" s="1">
         <v>46216</v>
       </c>
       <c r="M90" t="s">
@@ -3796,7 +3799,7 @@
         <v>226</v>
       </c>
     </row>
-    <row r="91" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A91" t="s">
         <v>264</v>
       </c>
@@ -3806,7 +3809,7 @@
       <c r="K91" t="s">
         <v>246</v>
       </c>
-      <c r="L91" s="2">
+      <c r="L91" s="1">
         <v>46216</v>
       </c>
       <c r="M91" t="s">
@@ -3819,7 +3822,7 @@
         <v>227</v>
       </c>
     </row>
-    <row r="92" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A92" t="s">
         <v>265</v>
       </c>
@@ -3829,7 +3832,7 @@
       <c r="K92" t="s">
         <v>246</v>
       </c>
-      <c r="L92" s="2">
+      <c r="L92" s="1">
         <v>46216</v>
       </c>
       <c r="M92" t="s">
@@ -3842,7 +3845,7 @@
         <v>228</v>
       </c>
     </row>
-    <row r="93" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A93" t="s">
         <v>266</v>
       </c>
@@ -3852,7 +3855,7 @@
       <c r="K93" t="s">
         <v>246</v>
       </c>
-      <c r="L93" s="2">
+      <c r="L93" s="1">
         <v>46216</v>
       </c>
       <c r="M93" t="s">
@@ -3865,7 +3868,7 @@
         <v>229</v>
       </c>
     </row>
-    <row r="94" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A94" t="s">
         <v>267</v>
       </c>
@@ -3875,7 +3878,7 @@
       <c r="K94" t="s">
         <v>246</v>
       </c>
-      <c r="L94" s="2">
+      <c r="L94" s="1">
         <v>46216</v>
       </c>
       <c r="M94" t="s">
@@ -3888,7 +3891,7 @@
         <v>230</v>
       </c>
     </row>
-    <row r="95" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A95" t="s">
         <v>268</v>
       </c>
@@ -3898,7 +3901,7 @@
       <c r="K95" t="s">
         <v>246</v>
       </c>
-      <c r="L95" s="2">
+      <c r="L95" s="1">
         <v>46216</v>
       </c>
       <c r="M95" t="s">
@@ -3911,7 +3914,7 @@
         <v>231</v>
       </c>
     </row>
-    <row r="96" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A96" t="s">
         <v>269</v>
       </c>
@@ -3921,7 +3924,7 @@
       <c r="K96" t="s">
         <v>246</v>
       </c>
-      <c r="L96" s="2">
+      <c r="L96" s="1">
         <v>46216</v>
       </c>
       <c r="M96" t="s">
@@ -3934,7 +3937,7 @@
         <v>232</v>
       </c>
     </row>
-    <row r="97" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A97" t="s">
         <v>270</v>
       </c>
@@ -3944,7 +3947,7 @@
       <c r="K97" t="s">
         <v>246</v>
       </c>
-      <c r="L97" s="2">
+      <c r="L97" s="1">
         <v>46216</v>
       </c>
       <c r="M97" t="s">
@@ -3957,7 +3960,7 @@
         <v>233</v>
       </c>
     </row>
-    <row r="98" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A98" t="s">
         <v>271</v>
       </c>
@@ -3967,7 +3970,7 @@
       <c r="K98" t="s">
         <v>246</v>
       </c>
-      <c r="L98" s="2">
+      <c r="L98" s="1">
         <v>46216</v>
       </c>
       <c r="M98" t="s">
@@ -3980,7 +3983,7 @@
         <v>234</v>
       </c>
     </row>
-    <row r="99" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A99" t="s">
         <v>272</v>
       </c>
@@ -3990,7 +3993,7 @@
       <c r="K99" t="s">
         <v>246</v>
       </c>
-      <c r="L99" s="2">
+      <c r="L99" s="1">
         <v>46216</v>
       </c>
       <c r="M99" t="s">
@@ -4003,7 +4006,7 @@
         <v>235</v>
       </c>
     </row>
-    <row r="100" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A100" t="s">
         <v>273</v>
       </c>
@@ -4013,7 +4016,7 @@
       <c r="K100" t="s">
         <v>246</v>
       </c>
-      <c r="L100" s="2">
+      <c r="L100" s="1">
         <v>46216</v>
       </c>
       <c r="M100" t="s">
@@ -4026,7 +4029,7 @@
         <v>236</v>
       </c>
     </row>
-    <row r="101" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A101" t="s">
         <v>274</v>
       </c>
@@ -4036,7 +4039,7 @@
       <c r="K101" t="s">
         <v>246</v>
       </c>
-      <c r="L101" s="2">
+      <c r="L101" s="1">
         <v>46216</v>
       </c>
       <c r="M101" t="s">
@@ -4049,7 +4052,7 @@
         <v>237</v>
       </c>
     </row>
-    <row r="102" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A102" t="s">
         <v>275</v>
       </c>
@@ -4059,7 +4062,7 @@
       <c r="K102" t="s">
         <v>246</v>
       </c>
-      <c r="L102" s="2">
+      <c r="L102" s="1">
         <v>46216</v>
       </c>
       <c r="M102" t="s">
@@ -4072,7 +4075,7 @@
         <v>238</v>
       </c>
     </row>
-    <row r="103" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A103" t="s">
         <v>276</v>
       </c>
@@ -4082,7 +4085,7 @@
       <c r="K103" t="s">
         <v>246</v>
       </c>
-      <c r="L103" s="2">
+      <c r="L103" s="1">
         <v>46216</v>
       </c>
       <c r="M103" t="s">
@@ -4095,7 +4098,7 @@
         <v>239</v>
       </c>
     </row>
-    <row r="104" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A104" t="s">
         <v>277</v>
       </c>
@@ -4105,7 +4108,7 @@
       <c r="K104" t="s">
         <v>246</v>
       </c>
-      <c r="L104" s="2">
+      <c r="L104" s="1">
         <v>46216</v>
       </c>
       <c r="M104" t="s">
@@ -4118,7 +4121,7 @@
         <v>240</v>
       </c>
     </row>
-    <row r="105" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A105" t="s">
         <v>278</v>
       </c>
@@ -4128,7 +4131,7 @@
       <c r="K105" t="s">
         <v>246</v>
       </c>
-      <c r="L105" s="2">
+      <c r="L105" s="1">
         <v>46216</v>
       </c>
       <c r="M105" t="s">
@@ -4141,7 +4144,7 @@
         <v>241</v>
       </c>
     </row>
-    <row r="106" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A106" t="s">
         <v>279</v>
       </c>
@@ -4151,7 +4154,7 @@
       <c r="K106" t="s">
         <v>246</v>
       </c>
-      <c r="L106" s="2">
+      <c r="L106" s="1">
         <v>46216</v>
       </c>
       <c r="M106" t="s">
@@ -4164,7 +4167,7 @@
         <v>242</v>
       </c>
     </row>
-    <row r="107" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A107" t="s">
         <v>280</v>
       </c>
@@ -4174,7 +4177,7 @@
       <c r="K107" t="s">
         <v>246</v>
       </c>
-      <c r="L107" s="2">
+      <c r="L107" s="1">
         <v>46216</v>
       </c>
       <c r="M107" t="s">
@@ -4187,7 +4190,7 @@
         <v>243</v>
       </c>
     </row>
-    <row r="108" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A108" t="s">
         <v>281</v>
       </c>
@@ -4197,7 +4200,7 @@
       <c r="K108" t="s">
         <v>246</v>
       </c>
-      <c r="L108" s="2">
+      <c r="L108" s="1">
         <v>46216</v>
       </c>
       <c r="M108" t="s">
@@ -4210,7 +4213,7 @@
         <v>244</v>
       </c>
     </row>
-    <row r="109" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A109" t="s">
         <v>282</v>
       </c>
@@ -4220,7 +4223,7 @@
       <c r="K109" t="s">
         <v>246</v>
       </c>
-      <c r="L109" s="2">
+      <c r="L109" s="1">
         <v>46216</v>
       </c>
       <c r="M109" t="s">
@@ -4233,7 +4236,7 @@
         <v>245</v>
       </c>
     </row>
-    <row r="110" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A110" t="s">
         <v>283</v>
       </c>
@@ -4243,7 +4246,7 @@
       <c r="K110" t="s">
         <v>355</v>
       </c>
-      <c r="L110" s="2">
+      <c r="L110" s="1">
         <v>46216</v>
       </c>
       <c r="M110" t="s">
@@ -4256,7 +4259,7 @@
         <v>319</v>
       </c>
     </row>
-    <row r="111" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A111" t="s">
         <v>284</v>
       </c>
@@ -4266,7 +4269,7 @@
       <c r="K111" t="s">
         <v>355</v>
       </c>
-      <c r="L111" s="2">
+      <c r="L111" s="1">
         <v>46216</v>
       </c>
       <c r="M111" t="s">
@@ -4279,7 +4282,7 @@
         <v>320</v>
       </c>
     </row>
-    <row r="112" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A112" t="s">
         <v>285</v>
       </c>
@@ -4289,7 +4292,7 @@
       <c r="K112" t="s">
         <v>355</v>
       </c>
-      <c r="L112" s="2">
+      <c r="L112" s="1">
         <v>46216</v>
       </c>
       <c r="M112" t="s">
@@ -4302,7 +4305,7 @@
         <v>321</v>
       </c>
     </row>
-    <row r="113" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="113" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A113" t="s">
         <v>286</v>
       </c>
@@ -4312,7 +4315,7 @@
       <c r="K113" t="s">
         <v>355</v>
       </c>
-      <c r="L113" s="2">
+      <c r="L113" s="1">
         <v>46216</v>
       </c>
       <c r="M113" t="s">
@@ -4325,7 +4328,7 @@
         <v>322</v>
       </c>
     </row>
-    <row r="114" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="114" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A114" t="s">
         <v>287</v>
       </c>
@@ -4335,7 +4338,7 @@
       <c r="K114" t="s">
         <v>355</v>
       </c>
-      <c r="L114" s="2">
+      <c r="L114" s="1">
         <v>46216</v>
       </c>
       <c r="M114" t="s">
@@ -4348,7 +4351,7 @@
         <v>323</v>
       </c>
     </row>
-    <row r="115" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="115" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A115" t="s">
         <v>288</v>
       </c>
@@ -4358,7 +4361,7 @@
       <c r="K115" t="s">
         <v>355</v>
       </c>
-      <c r="L115" s="2">
+      <c r="L115" s="1">
         <v>46216</v>
       </c>
       <c r="M115" t="s">
@@ -4371,7 +4374,7 @@
         <v>324</v>
       </c>
     </row>
-    <row r="116" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="116" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A116" t="s">
         <v>289</v>
       </c>
@@ -4381,7 +4384,7 @@
       <c r="K116" t="s">
         <v>355</v>
       </c>
-      <c r="L116" s="2">
+      <c r="L116" s="1">
         <v>46216</v>
       </c>
       <c r="M116" t="s">
@@ -4394,7 +4397,7 @@
         <v>325</v>
       </c>
     </row>
-    <row r="117" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="117" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A117" t="s">
         <v>290</v>
       </c>
@@ -4404,7 +4407,7 @@
       <c r="K117" t="s">
         <v>355</v>
       </c>
-      <c r="L117" s="2">
+      <c r="L117" s="1">
         <v>46216</v>
       </c>
       <c r="M117" t="s">
@@ -4417,7 +4420,7 @@
         <v>326</v>
       </c>
     </row>
-    <row r="118" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="118" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A118" t="s">
         <v>291</v>
       </c>
@@ -4427,7 +4430,7 @@
       <c r="K118" t="s">
         <v>355</v>
       </c>
-      <c r="L118" s="2">
+      <c r="L118" s="1">
         <v>46216</v>
       </c>
       <c r="M118" t="s">
@@ -4440,7 +4443,7 @@
         <v>327</v>
       </c>
     </row>
-    <row r="119" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="119" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A119" t="s">
         <v>292</v>
       </c>
@@ -4450,7 +4453,7 @@
       <c r="K119" t="s">
         <v>355</v>
       </c>
-      <c r="L119" s="2">
+      <c r="L119" s="1">
         <v>46216</v>
       </c>
       <c r="M119" t="s">
@@ -4463,7 +4466,7 @@
         <v>328</v>
       </c>
     </row>
-    <row r="120" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="120" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A120" t="s">
         <v>293</v>
       </c>
@@ -4473,7 +4476,7 @@
       <c r="K120" t="s">
         <v>355</v>
       </c>
-      <c r="L120" s="2">
+      <c r="L120" s="1">
         <v>46216</v>
       </c>
       <c r="M120" t="s">
@@ -4486,7 +4489,7 @@
         <v>329</v>
       </c>
     </row>
-    <row r="121" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="121" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A121" t="s">
         <v>294</v>
       </c>
@@ -4496,7 +4499,7 @@
       <c r="K121" t="s">
         <v>355</v>
       </c>
-      <c r="L121" s="2">
+      <c r="L121" s="1">
         <v>46216</v>
       </c>
       <c r="M121" t="s">
@@ -4509,7 +4512,7 @@
         <v>330</v>
       </c>
     </row>
-    <row r="122" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="122" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A122" t="s">
         <v>295</v>
       </c>
@@ -4519,7 +4522,7 @@
       <c r="K122" t="s">
         <v>355</v>
       </c>
-      <c r="L122" s="2">
+      <c r="L122" s="1">
         <v>46216</v>
       </c>
       <c r="M122" t="s">
@@ -4532,7 +4535,7 @@
         <v>331</v>
       </c>
     </row>
-    <row r="123" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="123" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A123" t="s">
         <v>296</v>
       </c>
@@ -4542,7 +4545,7 @@
       <c r="K123" t="s">
         <v>355</v>
       </c>
-      <c r="L123" s="2">
+      <c r="L123" s="1">
         <v>46216</v>
       </c>
       <c r="M123" t="s">
@@ -4555,7 +4558,7 @@
         <v>332</v>
       </c>
     </row>
-    <row r="124" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="124" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A124" t="s">
         <v>297</v>
       </c>
@@ -4565,7 +4568,7 @@
       <c r="K124" t="s">
         <v>355</v>
       </c>
-      <c r="L124" s="2">
+      <c r="L124" s="1">
         <v>46216</v>
       </c>
       <c r="M124" t="s">
@@ -4578,7 +4581,7 @@
         <v>333</v>
       </c>
     </row>
-    <row r="125" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="125" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A125" t="s">
         <v>298</v>
       </c>
@@ -4588,7 +4591,7 @@
       <c r="K125" t="s">
         <v>355</v>
       </c>
-      <c r="L125" s="2">
+      <c r="L125" s="1">
         <v>46216</v>
       </c>
       <c r="M125" t="s">
@@ -4601,7 +4604,7 @@
         <v>334</v>
       </c>
     </row>
-    <row r="126" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="126" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A126" t="s">
         <v>299</v>
       </c>
@@ -4611,7 +4614,7 @@
       <c r="K126" t="s">
         <v>355</v>
       </c>
-      <c r="L126" s="2">
+      <c r="L126" s="1">
         <v>46216</v>
       </c>
       <c r="M126" t="s">
@@ -4624,7 +4627,7 @@
         <v>335</v>
       </c>
     </row>
-    <row r="127" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="127" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A127" t="s">
         <v>300</v>
       </c>
@@ -4634,7 +4637,7 @@
       <c r="K127" t="s">
         <v>355</v>
       </c>
-      <c r="L127" s="2">
+      <c r="L127" s="1">
         <v>46216</v>
       </c>
       <c r="M127" t="s">
@@ -4647,7 +4650,7 @@
         <v>336</v>
       </c>
     </row>
-    <row r="128" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="128" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A128" t="s">
         <v>301</v>
       </c>
@@ -4657,7 +4660,7 @@
       <c r="K128" t="s">
         <v>355</v>
       </c>
-      <c r="L128" s="2">
+      <c r="L128" s="1">
         <v>46216</v>
       </c>
       <c r="M128" t="s">
@@ -4670,7 +4673,7 @@
         <v>337</v>
       </c>
     </row>
-    <row r="129" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="129" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A129" t="s">
         <v>302</v>
       </c>
@@ -4680,7 +4683,7 @@
       <c r="K129" t="s">
         <v>355</v>
       </c>
-      <c r="L129" s="2">
+      <c r="L129" s="1">
         <v>46216</v>
       </c>
       <c r="M129" t="s">
@@ -4693,7 +4696,7 @@
         <v>338</v>
       </c>
     </row>
-    <row r="130" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="130" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A130" t="s">
         <v>303</v>
       </c>
@@ -4703,7 +4706,7 @@
       <c r="K130" t="s">
         <v>355</v>
       </c>
-      <c r="L130" s="2">
+      <c r="L130" s="1">
         <v>46216</v>
       </c>
       <c r="M130" t="s">
@@ -4716,7 +4719,7 @@
         <v>339</v>
       </c>
     </row>
-    <row r="131" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="131" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A131" t="s">
         <v>304</v>
       </c>
@@ -4726,7 +4729,7 @@
       <c r="K131" t="s">
         <v>355</v>
       </c>
-      <c r="L131" s="2">
+      <c r="L131" s="1">
         <v>46216</v>
       </c>
       <c r="M131" t="s">
@@ -4739,7 +4742,7 @@
         <v>340</v>
       </c>
     </row>
-    <row r="132" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="132" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A132" t="s">
         <v>305</v>
       </c>
@@ -4749,7 +4752,7 @@
       <c r="K132" t="s">
         <v>355</v>
       </c>
-      <c r="L132" s="2">
+      <c r="L132" s="1">
         <v>46216</v>
       </c>
       <c r="M132" t="s">
@@ -4762,7 +4765,7 @@
         <v>341</v>
       </c>
     </row>
-    <row r="133" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="133" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A133" t="s">
         <v>306</v>
       </c>
@@ -4772,7 +4775,7 @@
       <c r="K133" t="s">
         <v>355</v>
       </c>
-      <c r="L133" s="2">
+      <c r="L133" s="1">
         <v>46216</v>
       </c>
       <c r="M133" t="s">
@@ -4785,7 +4788,7 @@
         <v>342</v>
       </c>
     </row>
-    <row r="134" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="134" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A134" t="s">
         <v>307</v>
       </c>
@@ -4795,7 +4798,7 @@
       <c r="K134" t="s">
         <v>355</v>
       </c>
-      <c r="L134" s="2">
+      <c r="L134" s="1">
         <v>46216</v>
       </c>
       <c r="M134" t="s">
@@ -4808,7 +4811,7 @@
         <v>343</v>
       </c>
     </row>
-    <row r="135" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="135" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A135" t="s">
         <v>308</v>
       </c>
@@ -4818,7 +4821,7 @@
       <c r="K135" t="s">
         <v>355</v>
       </c>
-      <c r="L135" s="2">
+      <c r="L135" s="1">
         <v>46216</v>
       </c>
       <c r="M135" t="s">
@@ -4831,7 +4834,7 @@
         <v>344</v>
       </c>
     </row>
-    <row r="136" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="136" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A136" t="s">
         <v>309</v>
       </c>
@@ -4841,7 +4844,7 @@
       <c r="K136" t="s">
         <v>355</v>
       </c>
-      <c r="L136" s="2">
+      <c r="L136" s="1">
         <v>46216</v>
       </c>
       <c r="M136" t="s">
@@ -4854,7 +4857,7 @@
         <v>345</v>
       </c>
     </row>
-    <row r="137" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="137" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A137" t="s">
         <v>310</v>
       </c>
@@ -4864,7 +4867,7 @@
       <c r="K137" t="s">
         <v>355</v>
       </c>
-      <c r="L137" s="2">
+      <c r="L137" s="1">
         <v>46216</v>
       </c>
       <c r="M137" t="s">
@@ -4877,7 +4880,7 @@
         <v>346</v>
       </c>
     </row>
-    <row r="138" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="138" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A138" t="s">
         <v>311</v>
       </c>
@@ -4887,7 +4890,7 @@
       <c r="K138" t="s">
         <v>355</v>
       </c>
-      <c r="L138" s="2">
+      <c r="L138" s="1">
         <v>46216</v>
       </c>
       <c r="M138" t="s">
@@ -4900,7 +4903,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="139" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="139" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A139" t="s">
         <v>312</v>
       </c>
@@ -4910,7 +4913,7 @@
       <c r="K139" t="s">
         <v>355</v>
       </c>
-      <c r="L139" s="2">
+      <c r="L139" s="1">
         <v>46216</v>
       </c>
       <c r="M139" t="s">
@@ -4923,7 +4926,7 @@
         <v>348</v>
       </c>
     </row>
-    <row r="140" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="140" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A140" t="s">
         <v>313</v>
       </c>
@@ -4933,7 +4936,7 @@
       <c r="K140" t="s">
         <v>355</v>
       </c>
-      <c r="L140" s="2">
+      <c r="L140" s="1">
         <v>46216</v>
       </c>
       <c r="M140" t="s">
@@ -4946,7 +4949,7 @@
         <v>349</v>
       </c>
     </row>
-    <row r="141" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="141" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A141" t="s">
         <v>314</v>
       </c>
@@ -4956,7 +4959,7 @@
       <c r="K141" t="s">
         <v>355</v>
       </c>
-      <c r="L141" s="2">
+      <c r="L141" s="1">
         <v>46216</v>
       </c>
       <c r="M141" t="s">
@@ -4969,7 +4972,7 @@
         <v>350</v>
       </c>
     </row>
-    <row r="142" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="142" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A142" t="s">
         <v>315</v>
       </c>
@@ -4979,7 +4982,7 @@
       <c r="K142" t="s">
         <v>355</v>
       </c>
-      <c r="L142" s="2">
+      <c r="L142" s="1">
         <v>46216</v>
       </c>
       <c r="M142" t="s">
@@ -4992,7 +4995,7 @@
         <v>351</v>
       </c>
     </row>
-    <row r="143" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="143" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A143" t="s">
         <v>316</v>
       </c>
@@ -5002,7 +5005,7 @@
       <c r="K143" t="s">
         <v>355</v>
       </c>
-      <c r="L143" s="2">
+      <c r="L143" s="1">
         <v>46216</v>
       </c>
       <c r="M143" t="s">
@@ -5015,7 +5018,7 @@
         <v>352</v>
       </c>
     </row>
-    <row r="144" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="144" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A144" t="s">
         <v>317</v>
       </c>
@@ -5025,7 +5028,7 @@
       <c r="K144" t="s">
         <v>355</v>
       </c>
-      <c r="L144" s="2">
+      <c r="L144" s="1">
         <v>46216</v>
       </c>
       <c r="M144" t="s">
@@ -5038,7 +5041,7 @@
         <v>353</v>
       </c>
     </row>
-    <row r="145" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="145" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A145" t="s">
         <v>318</v>
       </c>
@@ -5048,7 +5051,7 @@
       <c r="K145" t="s">
         <v>355</v>
       </c>
-      <c r="L145" s="2">
+      <c r="L145" s="1">
         <v>46216</v>
       </c>
       <c r="M145" t="s">
@@ -5061,7 +5064,7 @@
         <v>354</v>
       </c>
     </row>
-    <row r="146" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="146" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A146" t="s">
         <v>389</v>
       </c>
@@ -5069,9 +5072,9 @@
         <v>356</v>
       </c>
       <c r="K146" t="s">
-        <v>355</v>
-      </c>
-      <c r="L146" s="2">
+        <v>425</v>
+      </c>
+      <c r="L146" s="1">
         <v>46216</v>
       </c>
       <c r="M146" t="s">
@@ -5084,7 +5087,7 @@
         <v>356</v>
       </c>
     </row>
-    <row r="147" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="147" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A147" t="s">
         <v>390</v>
       </c>
@@ -5092,9 +5095,9 @@
         <v>357</v>
       </c>
       <c r="K147" t="s">
-        <v>355</v>
-      </c>
-      <c r="L147" s="2">
+        <v>425</v>
+      </c>
+      <c r="L147" s="1">
         <v>46216</v>
       </c>
       <c r="M147" t="s">
@@ -5107,7 +5110,7 @@
         <v>357</v>
       </c>
     </row>
-    <row r="148" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="148" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A148" t="s">
         <v>391</v>
       </c>
@@ -5115,9 +5118,9 @@
         <v>358</v>
       </c>
       <c r="K148" t="s">
-        <v>355</v>
-      </c>
-      <c r="L148" s="2">
+        <v>425</v>
+      </c>
+      <c r="L148" s="1">
         <v>46216</v>
       </c>
       <c r="M148" t="s">
@@ -5130,7 +5133,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="149" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="149" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A149" t="s">
         <v>392</v>
       </c>
@@ -5138,9 +5141,9 @@
         <v>359</v>
       </c>
       <c r="K149" t="s">
-        <v>355</v>
-      </c>
-      <c r="L149" s="2">
+        <v>425</v>
+      </c>
+      <c r="L149" s="1">
         <v>46216</v>
       </c>
       <c r="M149" t="s">
@@ -5153,7 +5156,7 @@
         <v>359</v>
       </c>
     </row>
-    <row r="150" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="150" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A150" t="s">
         <v>393</v>
       </c>
@@ -5161,9 +5164,9 @@
         <v>360</v>
       </c>
       <c r="K150" t="s">
-        <v>355</v>
-      </c>
-      <c r="L150" s="2">
+        <v>425</v>
+      </c>
+      <c r="L150" s="1">
         <v>46216</v>
       </c>
       <c r="M150" t="s">
@@ -5176,7 +5179,7 @@
         <v>360</v>
       </c>
     </row>
-    <row r="151" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="151" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A151" t="s">
         <v>394</v>
       </c>
@@ -5184,9 +5187,9 @@
         <v>361</v>
       </c>
       <c r="K151" t="s">
-        <v>355</v>
-      </c>
-      <c r="L151" s="2">
+        <v>425</v>
+      </c>
+      <c r="L151" s="1">
         <v>46216</v>
       </c>
       <c r="M151" t="s">
@@ -5199,7 +5202,7 @@
         <v>361</v>
       </c>
     </row>
-    <row r="152" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="152" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A152" t="s">
         <v>395</v>
       </c>
@@ -5207,9 +5210,9 @@
         <v>362</v>
       </c>
       <c r="K152" t="s">
-        <v>355</v>
-      </c>
-      <c r="L152" s="2">
+        <v>425</v>
+      </c>
+      <c r="L152" s="1">
         <v>46216</v>
       </c>
       <c r="M152" t="s">
@@ -5222,7 +5225,7 @@
         <v>362</v>
       </c>
     </row>
-    <row r="153" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="153" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A153" t="s">
         <v>396</v>
       </c>
@@ -5230,9 +5233,9 @@
         <v>363</v>
       </c>
       <c r="K153" t="s">
-        <v>355</v>
-      </c>
-      <c r="L153" s="2">
+        <v>425</v>
+      </c>
+      <c r="L153" s="1">
         <v>46216</v>
       </c>
       <c r="M153" t="s">
@@ -5245,7 +5248,7 @@
         <v>363</v>
       </c>
     </row>
-    <row r="154" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="154" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A154" t="s">
         <v>397</v>
       </c>
@@ -5253,9 +5256,9 @@
         <v>364</v>
       </c>
       <c r="K154" t="s">
-        <v>355</v>
-      </c>
-      <c r="L154" s="2">
+        <v>425</v>
+      </c>
+      <c r="L154" s="1">
         <v>46216</v>
       </c>
       <c r="M154" t="s">
@@ -5268,7 +5271,7 @@
         <v>364</v>
       </c>
     </row>
-    <row r="155" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="155" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A155" t="s">
         <v>398</v>
       </c>
@@ -5276,9 +5279,9 @@
         <v>365</v>
       </c>
       <c r="K155" t="s">
-        <v>355</v>
-      </c>
-      <c r="L155" s="2">
+        <v>425</v>
+      </c>
+      <c r="L155" s="1">
         <v>46216</v>
       </c>
       <c r="M155" t="s">
@@ -5291,7 +5294,7 @@
         <v>365</v>
       </c>
     </row>
-    <row r="156" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="156" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A156" t="s">
         <v>399</v>
       </c>
@@ -5299,9 +5302,9 @@
         <v>366</v>
       </c>
       <c r="K156" t="s">
-        <v>355</v>
-      </c>
-      <c r="L156" s="2">
+        <v>425</v>
+      </c>
+      <c r="L156" s="1">
         <v>46216</v>
       </c>
       <c r="M156" t="s">
@@ -5314,7 +5317,7 @@
         <v>366</v>
       </c>
     </row>
-    <row r="157" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="157" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A157" t="s">
         <v>400</v>
       </c>
@@ -5322,9 +5325,9 @@
         <v>367</v>
       </c>
       <c r="K157" t="s">
-        <v>355</v>
-      </c>
-      <c r="L157" s="2">
+        <v>425</v>
+      </c>
+      <c r="L157" s="1">
         <v>46216</v>
       </c>
       <c r="M157" t="s">
@@ -5337,7 +5340,7 @@
         <v>367</v>
       </c>
     </row>
-    <row r="158" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="158" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A158" t="s">
         <v>401</v>
       </c>
@@ -5345,9 +5348,9 @@
         <v>368</v>
       </c>
       <c r="K158" t="s">
-        <v>355</v>
-      </c>
-      <c r="L158" s="2">
+        <v>425</v>
+      </c>
+      <c r="L158" s="1">
         <v>46216</v>
       </c>
       <c r="M158" t="s">
@@ -5360,7 +5363,7 @@
         <v>368</v>
       </c>
     </row>
-    <row r="159" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="159" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A159" t="s">
         <v>402</v>
       </c>
@@ -5368,9 +5371,9 @@
         <v>369</v>
       </c>
       <c r="K159" t="s">
-        <v>355</v>
-      </c>
-      <c r="L159" s="2">
+        <v>425</v>
+      </c>
+      <c r="L159" s="1">
         <v>46216</v>
       </c>
       <c r="M159" t="s">
@@ -5383,7 +5386,7 @@
         <v>369</v>
       </c>
     </row>
-    <row r="160" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="160" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A160" t="s">
         <v>403</v>
       </c>
@@ -5391,9 +5394,9 @@
         <v>370</v>
       </c>
       <c r="K160" t="s">
-        <v>355</v>
-      </c>
-      <c r="L160" s="2">
+        <v>425</v>
+      </c>
+      <c r="L160" s="1">
         <v>46216</v>
       </c>
       <c r="M160" t="s">
@@ -5406,7 +5409,7 @@
         <v>370</v>
       </c>
     </row>
-    <row r="161" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="161" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A161" t="s">
         <v>404</v>
       </c>
@@ -5414,9 +5417,9 @@
         <v>371</v>
       </c>
       <c r="K161" t="s">
-        <v>355</v>
-      </c>
-      <c r="L161" s="2">
+        <v>425</v>
+      </c>
+      <c r="L161" s="1">
         <v>46216</v>
       </c>
       <c r="M161" t="s">
@@ -5429,7 +5432,7 @@
         <v>371</v>
       </c>
     </row>
-    <row r="162" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="162" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A162" t="s">
         <v>405</v>
       </c>
@@ -5437,9 +5440,9 @@
         <v>372</v>
       </c>
       <c r="K162" t="s">
-        <v>355</v>
-      </c>
-      <c r="L162" s="2">
+        <v>425</v>
+      </c>
+      <c r="L162" s="1">
         <v>46216</v>
       </c>
       <c r="M162" t="s">
@@ -5452,7 +5455,7 @@
         <v>372</v>
       </c>
     </row>
-    <row r="163" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="163" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A163" t="s">
         <v>406</v>
       </c>
@@ -5460,9 +5463,9 @@
         <v>373</v>
       </c>
       <c r="K163" t="s">
-        <v>355</v>
-      </c>
-      <c r="L163" s="2">
+        <v>425</v>
+      </c>
+      <c r="L163" s="1">
         <v>46216</v>
       </c>
       <c r="M163" t="s">
@@ -5475,7 +5478,7 @@
         <v>373</v>
       </c>
     </row>
-    <row r="164" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="164" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A164" t="s">
         <v>407</v>
       </c>
@@ -5483,9 +5486,9 @@
         <v>374</v>
       </c>
       <c r="K164" t="s">
-        <v>355</v>
-      </c>
-      <c r="L164" s="2">
+        <v>425</v>
+      </c>
+      <c r="L164" s="1">
         <v>46216</v>
       </c>
       <c r="M164" t="s">
@@ -5498,7 +5501,7 @@
         <v>374</v>
       </c>
     </row>
-    <row r="165" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="165" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A165" t="s">
         <v>408</v>
       </c>
@@ -5506,9 +5509,9 @@
         <v>375</v>
       </c>
       <c r="K165" t="s">
-        <v>355</v>
-      </c>
-      <c r="L165" s="2">
+        <v>425</v>
+      </c>
+      <c r="L165" s="1">
         <v>46216</v>
       </c>
       <c r="M165" t="s">
@@ -5521,7 +5524,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="166" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="166" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A166" t="s">
         <v>409</v>
       </c>
@@ -5529,9 +5532,9 @@
         <v>376</v>
       </c>
       <c r="K166" t="s">
-        <v>355</v>
-      </c>
-      <c r="L166" s="2">
+        <v>425</v>
+      </c>
+      <c r="L166" s="1">
         <v>46216</v>
       </c>
       <c r="M166" t="s">
@@ -5544,7 +5547,7 @@
         <v>376</v>
       </c>
     </row>
-    <row r="167" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="167" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A167" t="s">
         <v>410</v>
       </c>
@@ -5552,9 +5555,9 @@
         <v>377</v>
       </c>
       <c r="K167" t="s">
-        <v>355</v>
-      </c>
-      <c r="L167" s="2">
+        <v>425</v>
+      </c>
+      <c r="L167" s="1">
         <v>46216</v>
       </c>
       <c r="M167" t="s">
@@ -5567,7 +5570,7 @@
         <v>377</v>
       </c>
     </row>
-    <row r="168" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="168" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A168" t="s">
         <v>411</v>
       </c>
@@ -5575,9 +5578,9 @@
         <v>378</v>
       </c>
       <c r="K168" t="s">
-        <v>355</v>
-      </c>
-      <c r="L168" s="2">
+        <v>425</v>
+      </c>
+      <c r="L168" s="1">
         <v>46216</v>
       </c>
       <c r="M168" t="s">
@@ -5590,7 +5593,7 @@
         <v>378</v>
       </c>
     </row>
-    <row r="169" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="169" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A169" t="s">
         <v>412</v>
       </c>
@@ -5598,9 +5601,9 @@
         <v>379</v>
       </c>
       <c r="K169" t="s">
-        <v>355</v>
-      </c>
-      <c r="L169" s="2">
+        <v>425</v>
+      </c>
+      <c r="L169" s="1">
         <v>46216</v>
       </c>
       <c r="M169" t="s">
@@ -5613,7 +5616,7 @@
         <v>379</v>
       </c>
     </row>
-    <row r="170" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="170" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A170" t="s">
         <v>413</v>
       </c>
@@ -5621,9 +5624,9 @@
         <v>380</v>
       </c>
       <c r="K170" t="s">
-        <v>355</v>
-      </c>
-      <c r="L170" s="2">
+        <v>425</v>
+      </c>
+      <c r="L170" s="1">
         <v>46216</v>
       </c>
       <c r="M170" t="s">
@@ -5636,7 +5639,7 @@
         <v>380</v>
       </c>
     </row>
-    <row r="171" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="171" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A171" t="s">
         <v>414</v>
       </c>
@@ -5644,9 +5647,9 @@
         <v>381</v>
       </c>
       <c r="K171" t="s">
-        <v>355</v>
-      </c>
-      <c r="L171" s="2">
+        <v>425</v>
+      </c>
+      <c r="L171" s="1">
         <v>46216</v>
       </c>
       <c r="M171" t="s">
@@ -5659,7 +5662,7 @@
         <v>381</v>
       </c>
     </row>
-    <row r="172" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="172" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A172" t="s">
         <v>415</v>
       </c>
@@ -5667,9 +5670,9 @@
         <v>382</v>
       </c>
       <c r="K172" t="s">
-        <v>355</v>
-      </c>
-      <c r="L172" s="2">
+        <v>425</v>
+      </c>
+      <c r="L172" s="1">
         <v>46216</v>
       </c>
       <c r="M172" t="s">
@@ -5682,7 +5685,7 @@
         <v>382</v>
       </c>
     </row>
-    <row r="173" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="173" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A173" t="s">
         <v>416</v>
       </c>
@@ -5690,9 +5693,9 @@
         <v>383</v>
       </c>
       <c r="K173" t="s">
-        <v>355</v>
-      </c>
-      <c r="L173" s="2">
+        <v>425</v>
+      </c>
+      <c r="L173" s="1">
         <v>46216</v>
       </c>
       <c r="M173" t="s">
@@ -5705,7 +5708,7 @@
         <v>383</v>
       </c>
     </row>
-    <row r="174" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="174" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A174" t="s">
         <v>417</v>
       </c>
@@ -5713,9 +5716,9 @@
         <v>384</v>
       </c>
       <c r="K174" t="s">
-        <v>355</v>
-      </c>
-      <c r="L174" s="2">
+        <v>425</v>
+      </c>
+      <c r="L174" s="1">
         <v>46216</v>
       </c>
       <c r="M174" t="s">
@@ -5728,7 +5731,7 @@
         <v>384</v>
       </c>
     </row>
-    <row r="175" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="175" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A175" t="s">
         <v>418</v>
       </c>
@@ -5736,9 +5739,9 @@
         <v>385</v>
       </c>
       <c r="K175" t="s">
-        <v>355</v>
-      </c>
-      <c r="L175" s="2">
+        <v>425</v>
+      </c>
+      <c r="L175" s="1">
         <v>46216</v>
       </c>
       <c r="M175" t="s">
@@ -5751,7 +5754,7 @@
         <v>385</v>
       </c>
     </row>
-    <row r="176" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="176" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A176" t="s">
         <v>419</v>
       </c>
@@ -5759,9 +5762,9 @@
         <v>386</v>
       </c>
       <c r="K176" t="s">
-        <v>355</v>
-      </c>
-      <c r="L176" s="2">
+        <v>425</v>
+      </c>
+      <c r="L176" s="1">
         <v>46216</v>
       </c>
       <c r="M176" t="s">
@@ -5774,7 +5777,7 @@
         <v>386</v>
       </c>
     </row>
-    <row r="177" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="177" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A177" t="s">
         <v>420</v>
       </c>
@@ -5782,9 +5785,9 @@
         <v>387</v>
       </c>
       <c r="K177" t="s">
-        <v>355</v>
-      </c>
-      <c r="L177" s="2">
+        <v>425</v>
+      </c>
+      <c r="L177" s="1">
         <v>46216</v>
       </c>
       <c r="M177" t="s">
@@ -5797,7 +5800,7 @@
         <v>387</v>
       </c>
     </row>
-    <row r="178" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="178" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A178" t="s">
         <v>421</v>
       </c>
@@ -5805,9 +5808,9 @@
         <v>388</v>
       </c>
       <c r="K178" t="s">
-        <v>355</v>
-      </c>
-      <c r="L178" s="2">
+        <v>425</v>
+      </c>
+      <c r="L178" s="1">
         <v>46216</v>
       </c>
       <c r="M178" t="s">
@@ -5820,7 +5823,7 @@
         <v>388</v>
       </c>
     </row>
-    <row r="179" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="179" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A179" t="s">
         <v>422</v>
       </c>
@@ -5828,9 +5831,9 @@
         <v>74509</v>
       </c>
       <c r="K179" t="s">
-        <v>355</v>
-      </c>
-      <c r="L179" s="2">
+        <v>425</v>
+      </c>
+      <c r="L179" s="1">
         <v>46216</v>
       </c>
       <c r="M179" t="s">
@@ -5843,7 +5846,7 @@
         <v>74509</v>
       </c>
     </row>
-    <row r="180" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="180" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A180" t="s">
         <v>423</v>
       </c>
@@ -5851,9 +5854,9 @@
         <v>424</v>
       </c>
       <c r="K180" t="s">
-        <v>355</v>
-      </c>
-      <c r="L180" s="2">
+        <v>425</v>
+      </c>
+      <c r="L180" s="1">
         <v>46216</v>
       </c>
       <c r="M180" t="s">
@@ -5877,28 +5880,28 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:D29"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="25.875" customWidth="1"/>
-    <col min="2" max="2" width="12.875" customWidth="1"/>
-    <col min="3" max="3" width="45.875" customWidth="1"/>
-    <col min="4" max="4" width="30.875" customWidth="1"/>
+    <col min="1" max="1" width="25.83203125" customWidth="1"/>
+    <col min="2" max="2" width="12.83203125" customWidth="1"/>
+    <col min="3" max="3" width="45.83203125" customWidth="1"/>
+    <col min="4" max="4" width="30.83203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A1" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="B1" s="1"/>
-      <c r="C1" s="1"/>
-      <c r="D1" s="1"/>
-    </row>
-    <row r="2" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="B1" s="2"/>
+      <c r="C1" s="2"/>
+      <c r="D1" s="2"/>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="3" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>32</v>
       </c>
@@ -5906,12 +5909,12 @@
         <v>33</v>
       </c>
     </row>
-    <row r="4" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="5" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>34</v>
       </c>
@@ -5925,7 +5928,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="6" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>0</v>
       </c>
@@ -5939,7 +5942,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="7" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>1</v>
       </c>
@@ -5953,7 +5956,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="8" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>2</v>
       </c>
@@ -5967,7 +5970,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="9" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>3</v>
       </c>
@@ -5981,7 +5984,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="10" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>4</v>
       </c>
@@ -5995,7 +5998,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="11" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>5</v>
       </c>
@@ -6009,7 +6012,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="12" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>6</v>
       </c>
@@ -6023,7 +6026,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="13" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
         <v>7</v>
       </c>
@@ -6037,7 +6040,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="14" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
         <v>8</v>
       </c>
@@ -6051,7 +6054,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="15" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
         <v>9</v>
       </c>
@@ -6065,7 +6068,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="16" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
         <v>10</v>
       </c>
@@ -6079,7 +6082,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="17" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
         <v>11</v>
       </c>
@@ -6093,7 +6096,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="18" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
         <v>12</v>
       </c>
@@ -6107,7 +6110,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="19" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
         <v>13</v>
       </c>
@@ -6121,7 +6124,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="20" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
         <v>14</v>
       </c>
@@ -6135,12 +6138,12 @@
         <v>29</v>
       </c>
     </row>
-    <row r="21" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="22" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
         <v>56</v>
       </c>
@@ -6148,37 +6151,37 @@
         <v>31</v>
       </c>
     </row>
-    <row r="23" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="24" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="25" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="26" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
         <v>60</v>
       </c>
     </row>
-    <row r="27" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="28" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="29" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
         <v>63</v>
       </c>

</xml_diff>